<commit_message>
Invoice UI Refresh: reconcile suite to PRD v39 (non-substantive delta)
Re-supplied design + tech plan are identical to authoring inputs (design
content byte-identical; tech plan md5-identical). PRD moved v38->v39; the
only change is a Slack-channel link added to the header table plus one
trailing blank line removed -- no story/rule/wording change. No case
content changed. Re-stamped provenance v38->v39 (read date 25 Aug) on all
87 cases; regenerated import (87 rows, 0 shredded, one marker+provenance
each). Stored v39 body; refreshed Chris Ward PO-questions sheet (PO-2 now
names both un-logged edits, v39 verified cosmetic). Added reconcile note.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/testrail-import/Invoice-UI-Refresh_testrail-import.xlsx
+++ b/build/invoice-ui-refresh/testrail-import/Invoice-UI-Refresh_testrail-import.xlsx
@@ -518,7 +518,7 @@
 2. It shows the shop location's street address, city, state or province, postal code, and phone number.
 3. All of these identity details read exactly as they are entered for the shop location.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, section S1-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -569,7 +569,7 @@
           <t xml:space="preserve">1. When the shop has a logo set, the masthead shows that logo.
 2. When the shop has no logo set, the masthead shows no logo at all — and no placeholder image, box or 'no logo' text appears in its place.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, section S1-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -623,7 +623,7 @@
 3. The Credit Invoice label reads exactly "Credit: {number}", for example "Credit: CM-2202".
 4. In every case the number always includes its type prefix (EST-, INV-, or CM-), and the type word comes before the number.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, sections S1-R3 and S1-R4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, sections S1-R3 and S1-R4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -674,7 +674,7 @@
           <t xml:space="preserve">1. No status label or pill (for example "PAID", "PAID IN FULL", "DRAFT", "VOIDED") appears anywhere in the masthead of any document.
 2. The only place a status indicator appears is with the content that proves it: the Paid banner's pill (on portal-generated Invoice PDFs) and the Status column in the Credit Invoice's status table.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, section S1-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -728,7 +728,7 @@
 3. On the Invoice the boxed headline figure at the end of the totals block is labeled "Balance".
 4. The Credit Invoice has no boxed headline figure; its masthead carries only "Credit: {number}" and "Issue date: {date}", and its key figure (Total Credit) sits in the totals block.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, section S1-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -784,7 +784,7 @@
 4. The Credit Invoice masthead shows "Issue date: {date}".
 5. Every date reads in the fixed format, for example "Jan 5, 2026".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, sections S1-R7 and G-R1, read on 21 August 2026. The paid-date swap detail is in S10-R4 (see the Estimate and Invoice Specifics cases).
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, sections S1-R7 and G-R1, read on 25 August 2026. The paid-date swap detail is in S10-R4 (see the Estimate and Invoice Specifics cases).
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -835,7 +835,7 @@
           <t xml:space="preserve">1. Each missing field among the street address, city, state or province, postal code, and phone number is hidden — no blank line and no empty label is left where it would have been.
 2. The fields that do have values still show normally.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 38, section S1-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -887,7 +887,7 @@
 2. It shows the customer's name — the company name when the customer has one, otherwise the customer's personal name.
 3. It shows the customer's street address, city, state or province, and postal code.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 38, section S2-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -939,7 +939,7 @@
 2. The payee resolves from either mechanism: the shop's integrated-billing remit-to, or the location's own remit-to setting.
 3. The block appears on the Estimate and Invoice (not on the Credit Invoice).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 38, section S2-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -992,7 +992,7 @@
 2. When a Remit Payment To block is present, Bill To and Remit Payment To sit side by side.
 3. On the Credit Invoice, where Remit Payment To never appears, the Credit To block is always full width.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 38, section S2-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1043,7 +1043,7 @@
           <t xml:space="preserve">1. No "Remit Payment To" block is shown.
 2. The shop's own address is NOT printed as a fallback remit-to (this fallback has been removed).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 38, sections S2-N2 and S2-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, sections S2-N2 and S2-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1094,7 +1094,7 @@
           <t xml:space="preserve">1. Each missing field among the street address, city, state or province, and postal code is hidden — no blank line is left.
 2. The name line is always shown, even when the address fields are empty.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 38, section S2-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1146,7 +1146,7 @@
 2. Each field label has no punctuation after it (no colon).
 3. The labels read exactly as listed.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1198,7 +1198,7 @@
 2. When no terms are set, the field still shows: the text reads exactly "Terms" with an empty value area — no colon, and no placeholder text.
 3. Terms is the one order reference field that always shows (all others hide when empty).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, sections S3-R2 and S3-N4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, sections S3-R2 and S3-N4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1249,7 +1249,7 @@
           <t xml:space="preserve">1. The Authorizer field shows the full name of the work order's selected authorizer.
 2. The name matches the selected 'Approves Work' contact on the work order.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1300,7 +1300,7 @@
           <t xml:space="preserve">1. The Approval Code field shows the work order's integrated-billing approval code, in its own field labeled exactly "Approval Code".
 2. The approval code is no longer shown under the "Authorizer" label (net-new placement).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1352,7 +1352,7 @@
 2. When they differ, the Work Order field is shown with its value.
 3. Trailing digits example: "4176" in "INV-4176"; "24914" in "".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1405,7 +1405,7 @@
 3. The Approval Code field is hidden (no label, no empty value area).
 4. Terms still shows (it is the always-show exception).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, sections S3-N2, S3-N3 and S3-N5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, sections S3-N2, S3-N3 and S3-N5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1459,7 +1459,7 @@
 3. No other contact is offered, and no free-typed name can be entered.
 4. This is the only place the Authorizer can be selected.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1512,7 +1512,7 @@
 2. The Authorizer list includes a "No authorizer" option.
 3. Choosing "No authorizer" clears the selection back to empty.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1563,7 +1563,7 @@
           <t xml:space="preserve">1. When the selected authorizer's contact record has a phone number, the phone shows in the card directly below the authorizer's name, styled like the Contact's phone.
 2. When the contact record has no phone number, no phone row is shown under the authorizer's name.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R7, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R7, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1614,7 +1614,7 @@
           <t xml:space="preserve">1. Once the work order is invoiced, the Authorizer row is locked and its value cannot be changed.
 2. Before invoicing the row is editable; from the point of invoicing it is read-only.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R8, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R8, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1666,7 +1666,7 @@
           <t xml:space="preserve">1. The newly enabled contact appears in the work order's Authorizer list.
 2. It becomes selectable without any refresh or re-save of the work order.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 38, section S3-R9, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R9, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1719,7 +1719,7 @@
 3. When the asset has no VIN but has a serial number, the "VIN / Serial" value shows the serial number.
 4. The VIN is preferred when both exist.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 38, section S4-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1769,7 +1769,7 @@
         <is>
           <t xml:space="preserve">1. The asset section shows fields labeled exactly "Unit", "Plate", "Mileage", and "Eng Hrs" with their values.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 38, section S4-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1820,7 +1820,7 @@
           <t xml:space="preserve">1. Each of Unit, Plate, Mileage and Eng Hrs is hidden when it has no value — no blank label is left.
 2. The fields that do have values still show.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 38, section S4-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1871,7 +1871,7 @@
           <t xml:space="preserve">1. The "VIN / Serial" field is hidden when the asset has neither a VIN nor a serial number.
 2. The Asset name still shows.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 38, section S4-N2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-N2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1923,7 +1923,7 @@
           <t xml:space="preserve">1. The asset section shows whenever the work order has an asset attached — including on part sales, treated the same as service work orders.
 2. When the work order has no asset attached, the asset section is hidden entirely.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 38, sections S4-N3 and the Story 4 prerequisite, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, sections S4-N3 and the Story 4 prerequisite, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1974,7 +1974,7 @@
           <t xml:space="preserve">1. On the Estimate the work section heading reads exactly "Work Summary".
 2. On the Invoice the same section heading reads exactly "Work Performed".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, section S5-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2026,7 +2026,7 @@
 2. Lines 1 to 99 are zero-padded to two digits: 01, 02 ... 10, 11.
 3. When the document has 100 or more lines, lines 1-99 still show two digits and lines 100 and above show three digits (100, 101 ...).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, section S5-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2080,7 +2080,7 @@
 3. A line shows its scope-of-work note when a scope-of-work note is present (shown below the description).
 4. A line with no description and no scope-of-work note shows just its name (no empty rows).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, sections S5-R3, S5-R4 and S5-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, sections S5-R3, S5-R4 and S5-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2131,7 +2131,7 @@
           <t xml:space="preserve">1. A labor entry within a line is labeled exactly "Labor".
 2. A parts entry within a line is labeled exactly "Part" (singular).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, section S5-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2184,7 +2184,7 @@
 3. Turning "Labor price" off also hides the line footer's "Labor" figure; turning "Part price" off also hides the line footer's "Parts" figure.
 4. The itemized labor and parts entries themselves are never collapsed or hidden by any setting; "Line total" and the financial summary always show their amounts.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, section S5-R7, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R7, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2237,7 +2237,7 @@
 2. A discount that applies to a single line is shown with that line in parentheses (the accounting convention for a subtraction).
 3. The parentheses are required wording, not styling.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, section S5-R8, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R8, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2292,7 +2292,7 @@
 4. The vertical divider before "Line total" shows only when at least one Labor or Parts figure is visible; when neither is, "Line total" stands alone with no divider.
 5. "Line total" always shows, appears once per line, and shows even when it reads $0.00.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, sections S5-R7, S5-R9 and S5-R10, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, sections S5-R7, S5-R9 and S5-R10, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2343,7 +2343,7 @@
           <t xml:space="preserve">1. The work section shows its heading with no lines beneath it.
 2. The "Summary" divider still appears and precedes the financial summary.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 38, section S5-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2395,7 +2395,7 @@
 2. Each declined line shows its name, and its description when a description is present.
 3. A declined line never shows a scope-of-work note (the technician's internal write-up) - that note does not print for declined work on any customer document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 38, sections S6-R1 and S6-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 39, sections S6-R1 and S6-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2448,7 +2448,7 @@
 3. Declined lines do not show a line number.
 4. No status pill is shown on declined lines; the "Declined Work" heading is the only indicator of declined status.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 38, sections S6-R3, S6-R4 and S6-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 39, sections S6-R3, S6-R4 and S6-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2499,7 +2499,7 @@
           <t xml:space="preserve">1. When there are no declined lines, the Declined Work section is not shown.
 2. When the "Show declined work" option is off, the Declined Work section is not shown even if declined lines exist.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 38, section S6-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 39, section S6-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2549,7 +2549,7 @@
         <is>
           <t xml:space="preserve">1. A divider labeled exactly "Summary" precedes the financial summary.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 38, section S7-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, section S7-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2601,7 +2601,7 @@
 2. Each shows the gross amount - before any fees or discounts.
 3. A row labeled exactly "Shop supplies" shows only when a shop-supplies charge applies.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 38, sections S7-R2 and S7-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-R2 and S7-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2652,7 +2652,7 @@
           <t xml:space="preserve">1. When the location's "Show % on Estimates and Invoices" setting is enabled and shop supplies are charged as a percentage of labor, the percentage is shown alongside the shop supplies amount.
 2. Otherwise the shop supplies amount is shown alone.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 38, section S7-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, section S7-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2706,7 +2706,7 @@
 4. A work-order-wide discount shows in parentheses; a work-order-wide fee shows as a plain amount.
 5. There are intentionally two "Labor" rows and two "Parts" rows in the summary; the Adjustments pair is distinguished by sitting under the Adjustments heading.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 38, sections S7-R4 and S7-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-R4 and S7-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2760,7 +2760,7 @@
 4. Every row that contributes to the Subtotal is displayed; no contributing summary row is hidden.
 5. The visible math holds: gross Labor + gross Parts + Shop supplies + all Adjustments rows = Subtotal.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 38, sections S7-R7, S7-R8, S7-R9 and S7-R10, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-R7, S7-R8, S7-R9 and S7-R10, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2811,7 +2811,7 @@
           <t xml:space="preserve">1. The Adjustments heading is not shown when there is nothing to list under it (no work-order-wide fees or discounts and both rollup totals at zero).
 2. When no tax applies, no tax row is shown.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 38, sections S7-N1 and S7-N2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-N1 and S7-N2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2864,7 +2864,7 @@
 3. The amount shown is the applied amount when present, otherwise the payment amount.
 4. Rows list applied payments only, ordered by date; a fully reversed payment does not appear.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2916,7 +2916,7 @@
 2. When not configured, it shows the payment code with each underscore replaced by a space (for example credit_card shows as "credit card").
 3. The "SHOPPAY" code shows as "Online".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2967,7 +2967,7 @@
           <t xml:space="preserve">1. A deposit shows as a payment row labeled "(Deposit) {date} - {method}", where {date} is the date the deposit was collected.
 2. An applied customer-account credit shows as a payment row labeled "(Credit) {date} - {credit number}", where {credit number} is the full CM-prefixed number and {date} is the date the credit was applied.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-R4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3020,7 +3020,7 @@
 3. {full amount} is the payment's or deposit's full amount; {excess} is the full amount minus the amount applied to this invoice.
 4. The em dash and the arrow are literal separator characters, not subtraction.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3071,7 +3071,7 @@
 2. Balance equals the Total minus all applied payments (any method), applied deposits, and applied customer-account credits.
 3. Balance is floored at $0.00: an overpaid invoice shows "Balance" with "$0.00" - never a negative amount and never a hidden row.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3126,7 +3126,7 @@
 4. The banner shows a fixed status pill: exactly "PAID IN FULL" when the invoice is fully paid at generation time, otherwise exactly "PARTIALLY PAID".
 5. The banner title reads exactly "Payment Receipt (Batch) - Payments by ShopView" when every listed payment was part of a batch, otherwise exactly "Payment Receipt - Payments by ShopView".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-R8, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R8, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3181,7 +3181,7 @@
 5. In a batch, each payment carries a "Payment X of Y - Batch" marker.
 6. "Date / Time" reads in the format "Jan 5, 2026 - 2:41 PM MST" (date, then time with timezone).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, sections S8-R9 and G-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, sections S8-R9 and G-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3232,7 +3232,7 @@
           <t xml:space="preserve">1. A payment row whose amount is $0.00 is not shown.
 2. When no payments, deposits or customer-account credits have been applied, the Payments heading shows with no rows and the Balance equals the Total.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, sections S8-R7 and S8-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, sections S8-R7 and S8-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3283,7 +3283,7 @@
           <t xml:space="preserve">1. When the invoice has no portal-processed payment, the paid banner is not shown - a shop-recorded payment never produces the banner.
 2. An Invoice PDF generated in the shop app shows no banner in any case.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 38, section S8-N2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-N2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3334,7 +3334,7 @@
           <t xml:space="preserve">1. Each document shows the shop's configured disclaimer text, with no heading above it.
 2. The disclaimer is identical on every document that carries it.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 38, section S9-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, section S9-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3386,7 +3386,7 @@
 2. The three lines are identical on every document that carries the area.
 3. The signature area contains no authorization or acknowledgment sentence - only the three lines.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 38, sections S9-R2 and S9-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, sections S9-R2 and S9-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3437,7 +3437,7 @@
           <t xml:space="preserve">1. The footer shows the shop's tax identifier exactly as the shop entered it.
 2. No label is added in front of it (the shop types its own label into the field).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 38, section S9-R4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, section S9-R4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3488,7 +3488,7 @@
           <t xml:space="preserve">1. When the shop has no configured disclaimer, the disclaimer area is not shown.
 2. When the shop has no tax identifier configured, the footer tax identifier is not shown.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 38, sections S9-N1 and S9-N2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, sections S9-N1 and S9-N2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3538,7 +3538,7 @@
         <is>
           <t xml:space="preserve">1. The Estimate and Invoice carry the same content, differing only in: the document label, the dates, the work-section heading, the headline figure label, and the presence of the Paid banner and the Payments and Balance sections on the Invoice.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 38, section S10-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3592,7 +3592,7 @@
 4. No validity or expiry date is shown; no due-date line is shown.
 5. The signature area's "Date" line is unaffected.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 38, section S10-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3644,7 +3644,7 @@
 2. The boxed headline figure is labeled "Balance".
 3. The masthead shows "Invoice date: {date}" and "Due date: {date}".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 38, section S10-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3698,7 +3698,7 @@
 4. If a later change (payment reversal, voided credit, or edit) makes the Balance greater than $0.00, the invoice is no longer fully paid and "Due date: {date}" returns.
 5. A paid date earlier than the invoice date (for example a deposit collected before invoicing) is shown as-is.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 38, section S10-R4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3749,7 +3749,7 @@
           <t xml:space="preserve">1. An Invoice with no due date set shows "Invoice date: {date}" and no "Due date" line (the old quirk of rendering a null due date as today's date is retired).
 2. When such an invoice becomes fully paid, "Paid date: {date}" is shown.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 38, section S10-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3801,7 +3801,7 @@
 2. The masthead shows "Issue date: {date}".
 3. The masthead shows no money figure and no boxed headline figure.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, sections S11-R1 and S1-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R1 and S1-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3853,7 +3853,7 @@
 2. Every other address rule applies to it unchanged (name always shown, address fields hide when empty).
 3. Remit Payment To never appears on the Credit Invoice, so the Credit To block is always full width.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, sections S11-R2, S2-R1 and S2-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R2, S2-R1 and S2-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3906,7 +3906,7 @@
 3. Invoice Number shows the originating invoice's full document number (for example "").
 4. For an account-level credit with no origin invoice, the whole Invoice Number column is hidden.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, section S11-R3, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, section S11-R3, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3961,7 +3961,7 @@
 5. Totals are negative, formatted with a leading minus (for example "-$100.00") - not the parentheses convention used for discounts.
 6. A money-only line's Description comes from the credit's reason if entered, otherwise the memo text, otherwise "Refund".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, sections S11-R4 and S11-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R4 and S11-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4012,7 +4012,7 @@
           <t xml:space="preserve">1. The restocking fee reduces the credit: quantity -2 at rate $50.00 with a $10.00 restocking fee produces Total -$90.00.
 2. For a money-only line, Total is the credited amount.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, section S11-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, section S11-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4067,7 +4067,7 @@
 5. Refunded: one row per refund payment reading "{date} - {method}" with the refunded amount (negative); Balance reads $0.00 once fully consumed, otherwise the open balance, positive.
 6. Voided: Payments shows the label with no rows; Balance reads $0.00.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, sections S11-R6 and S11-R6a, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R6 and S11-R6a, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4118,7 +4118,7 @@
           <t xml:space="preserve">1. The Credit Invoice shows the shop's configured disclaimer.
 2. It shows the standard signature area with the three lines "Customer Signature", "Printed Name", and "Date".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 38, sections S11-R7 and S9-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R7 and S9-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4168,7 +4168,7 @@
         <is>
           <t xml:space="preserve">1. The document layout follows the Design Document exactly: masthead with the shop letterhead left, the shop logo center, and the document block right over a 2px ink rule; a bordered Addresses row; the asset band; the order reference chips; numbered work lines; the "Summary" break bar; a two-column tail with the disclaimer left and the totals right; the boxed headline figure; the three-line signature row; the single-line footer.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R1, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R1, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4219,7 +4219,7 @@
           <t xml:space="preserve">1. The only colours on any document are: ink #121926, body text #364152, muted text #697586, faint labels #9AA4B2, hairlines #E3E8EF, row dividers #EEF2F6, accent #257CFF, negative #B42318, paper #FFFFFF.
 2. No colour outside this closed set appears.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R2, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R2, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4270,7 +4270,7 @@
           <t xml:space="preserve">1. The accent #257CFF appears only on the work line numbers and on the word "ShopView" in the footer.
 2. Nothing else on the document uses the accent.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R3, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R3, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4322,7 +4322,7 @@
 2. Weight 400 for body text; 600 and 700 for emphasis and totals; 750 for the in-job section labels; 800 for the shop name, the document label, the headline figure, and the line numbers.
 3. Uppercase micro-labels carry letterspacing as in the Design Document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R4, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R4, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4374,7 +4374,7 @@
 2. Text smaller than 10px renders no lighter than #364152.
 3. Hairline rules render no lighter than #CDD5DF.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R5, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R5, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4425,7 +4425,7 @@
           <t xml:space="preserve">1. Every document is fully legible printed in grayscale.
 2. Colour is never the only signal: credit amounts also carry the leading minus, and discounts also carry parentheses.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R6, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R6, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4477,7 +4477,7 @@
 2. Only the white sheet is the document.
 3. The PDF output carries no drop shadow and no rounded sheet corners (those are screen-prototype presentation only).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, sections S12-R7 and S12-N1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, sections S12-R7 and S12-N1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4531,7 +4531,7 @@
 4. The "Labor" and "Parts" sub-section labels carry no underline rule.
 5. When a line has fee or discount adjustment rows, the row divider follows the line's last adjustment row - never between the line and its adjustments - so the line and its adjustments read as one group.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R8, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R8, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4584,7 +4584,7 @@
 3. The in-job "Labor" and "Parts" labels are 10.5px weight 750 in full ink #121926.
 4. All three sit visually below the 16px weight-700 job titles, with letterspacing per the Design Document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 38, section S12-R9, and the Design Document, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R9, and the Design Document, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4634,7 +4634,7 @@
         <is>
           <t xml:space="preserve">1. The Parts Sale Estimate behaves as the Estimate, and the Parts Sale Invoice as the Invoice, throughout the spec: masthead and date labels (including "Estimate date" and the Due/Paid date swap), addresses and Remit Payment To, asset section, financial summary, payments and Balance, the paid banner rule, disclaimer and signature, and the visual standard - except as Story 13 states.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-R1, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R1, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4686,7 +4686,7 @@
 2. It shows flat part lines, each with part number, description, quantity, rate, and amount.
 3. There are no job blocks, no "Scope of work", no Labor section, and no Declined Work section on a parts sale document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-R2, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R2, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4737,7 +4737,7 @@
           <t xml:space="preserve">1. Line-level fees and discounts render exactly as on the Invoice: indented under their part line.
 2. The row divider follows the part's last adjustment row, rather than sitting between the part and its adjustments.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, sections S13-R3 and S12-R8, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, sections S13-R3 and S12-R8, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4788,7 +4788,7 @@
           <t xml:space="preserve">1. The document number uses the parts-sale numbering through the existing document numbering.
 2. For example the Estimate reads "Estimate: EST-P2-1088" and the Invoice reads "Invoice: INV-P2-1088".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-R4, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R4, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4840,7 +4840,7 @@
 2. Customer PO and Terms are unchanged (Terms always shows).
 3. Authorizer follows the parts-sale Authorizer treatment (S13-R6).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-R5, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R5, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4893,7 +4893,7 @@
 2. It is locked once the parts sale is invoiced.
 3. When set, the authorizer's name prints in the document's Authorizer reference field.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-R6, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R6, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4944,7 +4944,7 @@
           <t xml:space="preserve">1. The financial summary shows no "Labor" row and no "Shop supplies" row.
 2. The "Parts" row, the adjustment rows, "Subtotal", "Tax", "Total", "Payments", and "Balance" are identical to the Invoice.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-R7, read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R7, read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4996,7 +4996,7 @@
 2. They keep their current templates until the follow-up ticket (SV-9193) ships.
 3. Restyling shared template partials must not half-restyle these deferred templates.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 38, section S13-N1, and story SV-9193 (deferred), read on 21 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-N1, and story SV-9193 (deferred), read on 25 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>

</xml_diff>

<commit_message>
Invoice UI Refresh: push v45 cases to TestRail, backfill id-map, sync R417
update_case on 87 (block-only HTML via to_ol/expected_html, render self-check green
on all 89), add_case INV-VIS-10->C45213 and INV-VIS-11->C45214 into section 6753,
id-map backfilled 89/89, run R417 union-synced 117->119 tests (union-only, Rule 34;
30 foreign creator-6 cases already present were preserved, 2 ours added).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QvLHRX1rY5c7HuyoMWVGpU
</commit_message>
<xml_diff>
--- a/build/invoice-ui-refresh/testrail-import/Invoice-UI-Refresh_testrail-import.xlsx
+++ b/build/invoice-ui-refresh/testrail-import/Invoice-UI-Refresh_testrail-import.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -518,7 +518,7 @@
 2. It shows the shop location's street address, city, state or province, postal code, and phone number.
 3. All of these identity details read exactly as they are entered for the shop location.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, section S1-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -569,7 +569,7 @@
           <t xml:space="preserve">1. When the shop has a logo set, the masthead shows that logo.
 2. When the shop has no logo set, the masthead shows no logo at all — and no placeholder image, box or 'no logo' text appears in its place.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, section S1-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -623,7 +623,7 @@
 3. The Credit Invoice label reads exactly "Credit: {number}", for example "Credit: CM-2202".
 4. In every case the number always includes its type prefix (EST-, INV-, or CM-), and the type word comes before the number.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, sections S1-R3 and S1-R4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, sections S1-R3 and S1-R4, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -674,7 +674,7 @@
           <t xml:space="preserve">1. No status label or pill (for example "PAID", "PAID IN FULL", "DRAFT", "VOIDED") appears anywhere in the masthead of any document.
 2. The only place a status indicator appears is with the content that proves it: the Paid banner's pill (on portal-generated Invoice PDFs) and the Status column in the Credit Invoice's status table.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, section S1-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -728,7 +728,7 @@
 3. On the Invoice the boxed headline figure at the end of the totals block is labeled "Balance".
 4. The Credit Invoice has no boxed headline figure; its masthead carries only "Credit: {number}" and "Issue date: {date}", and its key figure (Total Credit) sits in the totals block.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-R6, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, section S1-R6, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -784,7 +784,7 @@
 4. The Credit Invoice masthead shows "Issue date: {date}".
 5. Every date reads in the fixed format, for example "Jan 5, 2026".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, sections S1-R7 and G-R1, read on 25 August 2026. The paid-date swap detail is in S10-R4 (see the Estimate and Invoice Specifics cases).
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, sections S1-R7 and G-R1, read on 31 August 2026. The paid-date swap detail is in S10-R4 (see the Estimate and Invoice Specifics cases).
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -835,7 +835,7 @@
           <t xml:space="preserve">1. Each missing field among the street address, city, state or province, postal code, and phone number is hidden — no blank line and no empty label is left where it would have been.
 2. The fields that do have values still show normally.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 39, section S1-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9140 (Story 1, Masthead and Letterhead) and the Invoice UI Refresh specification version 45, section S1-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -887,7 +887,7 @@
 2. It shows the customer's name — the company name when the customer has one, otherwise the customer's personal name.
 3. It shows the customer's street address, city, state or province, and postal code.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 45, section S2-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -939,7 +939,7 @@
 2. The payee resolves from either mechanism: the shop's integrated-billing remit-to, or the location's own remit-to setting.
 3. The block appears on the Estimate and Invoice (not on the Credit Invoice).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 45, section S2-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -992,7 +992,7 @@
 2. When a Remit Payment To block is present, Bill To and Remit Payment To sit side by side.
 3. On the Credit Invoice, where Remit Payment To never appears, the Credit To block is always full width.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 45, section S2-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1043,7 +1043,7 @@
           <t xml:space="preserve">1. No "Remit Payment To" block is shown.
 2. The shop's own address is NOT printed as a fallback remit-to (this fallback has been removed).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, sections S2-N2 and S2-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 45, sections S2-N2 and S2-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1094,7 +1094,7 @@
           <t xml:space="preserve">1. Each missing field among the street address, city, state or province, and postal code is hidden — no blank line is left.
 2. The name line is always shown, even when the address fields are empty.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 39, section S2-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9141 (Story 2, Addresses) and the Invoice UI Refresh specification version 45, section S2-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1146,7 +1146,7 @@
 2. Each field label has no punctuation after it (no colon).
 3. The labels read exactly as listed.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1198,7 +1198,7 @@
 2. When no terms are set, the field still shows: the text reads exactly "Terms" with an empty value area — no colon, and no placeholder text.
 3. Terms is the one order reference field that always shows (all others hide when empty).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, sections S3-R2 and S3-N4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, sections S3-R2 and S3-N4, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1249,7 +1249,7 @@
           <t xml:space="preserve">1. The Authorizer field shows the full name of the work order's selected authorizer.
 2. The name matches the selected 'Approves Work' contact on the work order.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1300,7 +1300,7 @@
           <t xml:space="preserve">1. The Approval Code field shows the work order's integrated-billing approval code, in its own field labeled exactly "Approval Code".
 2. The approval code is no longer shown under the "Authorizer" label (net-new placement).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R4, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1352,7 +1352,7 @@
 2. When they differ, the Work Order field is shown with its value.
 3. Trailing digits example: "4176" in "INV-4176"; "24914" in "".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1405,7 +1405,7 @@
 3. The Approval Code field is hidden (no label, no empty value area).
 4. Terms still shows (it is the always-show exception).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, sections S3-N2, S3-N3 and S3-N5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, sections S3-N2, S3-N3 and S3-N5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1459,7 +1459,7 @@
 3. No other contact is offered, and no free-typed name can be entered.
 4. This is the only place the Authorizer can be selected.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1512,7 +1512,7 @@
 2. The Authorizer list includes a "No authorizer" option.
 3. Choosing "No authorizer" clears the selection back to empty.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R6, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R6, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1563,7 +1563,7 @@
           <t xml:space="preserve">1. When the selected authorizer's contact record has a phone number, the phone shows in the card directly below the authorizer's name, styled like the Contact's phone.
 2. When the contact record has no phone number, no phone row is shown under the authorizer's name.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R7, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R7, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1613,8 +1613,9 @@
         <is>
           <t xml:space="preserve">1. Once the work order is invoiced, the Authorizer row is locked and its value cannot be changed.
 2. Before invoicing the row is editable; from the point of invoicing it is read-only.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R8, read on 25 August 2026.
+3. If the invoice is later voided or reversed, the work order returns to Complete and the Authorizer row is re-enabled.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R8, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1666,7 +1667,7 @@
           <t xml:space="preserve">1. The newly enabled contact appears in the work order's Authorizer list.
 2. It becomes selectable without any refresh or re-save of the work order.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 39, section S3-R9, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9142 (Story 3, Order Reference Fields) and the Invoice UI Refresh specification version 45, section S3-R9, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1719,7 +1720,7 @@
 3. When the asset has no VIN but has a serial number, the "VIN / Serial" value shows the serial number.
 4. The VIN is preferred when both exist.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 45, section S4-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1769,7 +1770,7 @@
         <is>
           <t xml:space="preserve">1. The asset section shows fields labeled exactly "Unit", "Plate", "Mileage", and "Eng Hrs" with their values.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 45, section S4-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1820,7 +1821,7 @@
           <t xml:space="preserve">1. Each of Unit, Plate, Mileage and Eng Hrs is hidden when it has no value — no blank label is left.
 2. The fields that do have values still show.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 45, section S4-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1871,7 +1872,7 @@
           <t xml:space="preserve">1. The "VIN / Serial" field is hidden when the asset has neither a VIN nor a serial number.
 2. The Asset name still shows.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, section S4-N2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 45, section S4-N2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1923,7 +1924,7 @@
           <t xml:space="preserve">1. The asset section shows whenever the work order has an asset attached — including on part sales, treated the same as service work orders.
 2. When the work order has no asset attached, the asset section is hidden entirely.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 39, sections S4-N3 and the Story 4 prerequisite, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9143 (Story 4, Asset Section) and the Invoice UI Refresh specification version 45, sections S4-N3 and the Story 4 prerequisite, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -1974,7 +1975,7 @@
           <t xml:space="preserve">1. On the Estimate the work section heading reads exactly "Work Summary".
 2. On the Invoice the same section heading reads exactly "Work Performed".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, section S5-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2026,7 +2027,7 @@
 2. Lines 1 to 99 are zero-padded to two digits: 01, 02 ... 10, 11.
 3. When the document has 100 or more lines, lines 1-99 still show two digits and lines 100 and above show three digits (100, 101 ...).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, section S5-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2080,7 +2081,7 @@
 3. A line shows its scope-of-work note when a scope-of-work note is present (shown below the description).
 4. A line with no description and no scope-of-work note shows just its name (no empty rows).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, sections S5-R3, S5-R4 and S5-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, sections S5-R3, S5-R4 and S5-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2096,7 +2097,7 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>Labor and Part entries are labeled exactly 'Labor' and 'Part'</t>
+          <t>Labor and Parts entries are labeled exactly 'Labor' and 'Parts'</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
@@ -2129,9 +2130,9 @@
       <c r="G33" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. A labor entry within a line is labeled exactly "Labor".
-2. A parts entry within a line is labeled exactly "Part" (singular).
----
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R6, read on 25 August 2026.
+2. A parts entry within a line is labeled exactly "Parts".
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, section S5-R6, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2173,18 +2174,18 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>1. Under Administration &gt; Invoice Details, turn each of "Labor hours", "Labor rate", "Labor price", "Part quantity", "Part price" on, generate a document, and read a work line.
+          <t>1. Under Administration &gt; Invoice Details, turn each of "Labor hours", "Labor rate", "Labor price", "Part quantity", "Part price", "Part number" and "Part description" on, generate a document, and read a work line.
 2. Turn each setting off, generate again, and read the same line.</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. When "Labor hours", "Labor rate", "Labor price", "Part quantity" and "Part price" are on, each figure shows on its labor/part entry.
-2. Turning a setting off hides its per-entry figure.
+          <t xml:space="preserve">1. When "Labor hours", "Labor rate", "Labor price", "Part quantity", "Part price", "Part number" and "Part description" are on, each per-entry figure, the part number, and the part description show on their labor/part entry.
+2. Turning a setting off hides its per-entry figure; turning "Part number" off hides the part number on every parts entry, and turning "Part description" off hides the part description on every parts entry.
 3. Turning "Labor price" off also hides the line footer's "Labor" figure; turning "Part price" off also hides the line footer's "Parts" figure.
 4. The itemized labor and parts entries themselves are never collapsed or hidden by any setting; "Line total" and the financial summary always show their amounts.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R7, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, section S5-R7, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2237,7 +2238,7 @@
 2. A discount that applies to a single line is shown with that line in parentheses (the accounting convention for a subtraction).
 3. The parentheses are required wording, not styling.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-R8, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, section S5-R8, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2292,7 +2293,7 @@
 4. The vertical divider before "Line total" shows only when at least one Labor or Parts figure is visible; when neither is, "Line total" stands alone with no divider.
 5. "Line total" always shows, appears once per line, and shows even when it reads $0.00.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, sections S5-R7, S5-R9 and S5-R10, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, sections S5-R7, S5-R9 and S5-R10, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2343,7 +2344,7 @@
           <t xml:space="preserve">1. The work section shows its heading with no lines beneath it.
 2. The "Summary" divider still appears and precedes the financial summary.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 39, section S5-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9144 (Story 5, Work Section) and the Invoice UI Refresh specification version 45, section S5-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2395,7 +2396,7 @@
 2. Each declined line shows its name, and its description when a description is present.
 3. A declined line never shows a scope-of-work note (the technician's internal write-up) - that note does not print for declined work on any customer document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 39, sections S6-R1 and S6-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 45, sections S6-R1 and S6-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2448,7 +2449,7 @@
 3. Declined lines do not show a line number.
 4. No status pill is shown on declined lines; the "Declined Work" heading is the only indicator of declined status.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 39, sections S6-R3, S6-R4 and S6-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 45, sections S6-R3, S6-R4 and S6-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2499,7 +2500,7 @@
           <t xml:space="preserve">1. When there are no declined lines, the Declined Work section is not shown.
 2. When the "Show declined work" option is off, the Declined Work section is not shown even if declined lines exist.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 39, section S6-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9145 (Story 6, Declined Work) and the Invoice UI Refresh specification version 45, section S6-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2549,7 +2550,7 @@
         <is>
           <t xml:space="preserve">1. A divider labeled exactly "Summary" precedes the financial summary.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, section S7-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 45, section S7-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2601,7 +2602,7 @@
 2. Each shows the gross amount - before any fees or discounts.
 3. A row labeled exactly "Shop supplies" shows only when a shop-supplies charge applies.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-R2 and S7-R6, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 45, sections S7-R2 and S7-R6, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2652,7 +2653,7 @@
           <t xml:space="preserve">1. When the location's "Show % on Estimates and Invoices" setting is enabled and shop supplies are charged as a percentage of labor, the percentage is shown alongside the shop supplies amount.
 2. Otherwise the shop supplies amount is shown alone.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, section S7-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 45, section S7-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2706,7 +2707,7 @@
 4. A work-order-wide discount shows in parentheses; a work-order-wide fee shows as a plain amount.
 5. There are intentionally two "Labor" rows and two "Parts" rows in the summary; the Adjustments pair is distinguished by sitting under the Adjustments heading.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-R4 and S7-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 45, sections S7-R4 and S7-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2760,7 +2761,7 @@
 4. Every row that contributes to the Subtotal is displayed; no contributing summary row is hidden.
 5. The visible math holds: gross Labor + gross Parts + Shop supplies + all Adjustments rows = Subtotal.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-R7, S7-R8, S7-R9 and S7-R10, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 45, sections S7-R7, S7-R8, S7-R9 and S7-R10, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2811,7 +2812,7 @@
           <t xml:space="preserve">1. The Adjustments heading is not shown when there is nothing to list under it (no work-order-wide fees or discounts and both rollup totals at zero).
 2. When no tax applies, no tax row is shown.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 39, sections S7-N1 and S7-N2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9146 (Story 7, Financial Summary) and the Invoice UI Refresh specification version 45, sections S7-N1 and S7-N2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2862,9 +2863,9 @@
           <t xml:space="preserve">1. The Invoice shows a heading labeled exactly "Payments".
 2. Each applied payment shows as a row reading "{date} - {method}" (for example "Jul 30, 2026 - Cash"), where the hyphen is a literal character.
 3. The amount shown is the applied amount when present, otherwise the payment amount.
-4. Rows list applied payments only, ordered by date; a fully reversed payment does not appear.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R2, read on 25 August 2026.
+4. Rows list applied payments only, ordered by date and then by the order the payments were recorded; a fully reversed payment does not appear.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2916,7 +2917,7 @@
 2. When not configured, it shows the payment code with each underscore replaced by a space (for example credit_card shows as "credit card").
 3. The "SHOPPAY" code shows as "Online".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -2967,7 +2968,7 @@
           <t xml:space="preserve">1. A deposit shows as a payment row labeled "(Deposit) {date} - {method}", where {date} is the date the deposit was collected.
 2. An applied customer-account credit shows as a payment row labeled "(Credit) {date} - {credit number}", where {credit number} is the full CM-prefixed number and {date} is the date the credit was applied.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-R4, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3004,23 +3005,24 @@
       <c r="E50" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
-2. An Invoice has a payment (or deposit) whose amount exceeds the amount applied to this invoice - one where the excess became a numbered credit, and one where it has not yet.</t>
+2. An Invoice has a payment or deposit whose amount applied to this invoice is less than its full amount - for example an over-collected deposit, or a regular payment spread across more than one invoice - with one case where the excess became a numbered credit and one where it has not yet.</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
           <t>1. Generate the Invoice.
-2. Read the sub-line beneath the over-applied payment or deposit row.</t>
+2. Read the sub-line beneath the row whose applied amount is less than its full amount (payment or deposit).</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. When the excess has become a customer-account credit with a number, the sub-line reads exactly "of {full amount} - {excess} -&gt; Credit {credit number}" (for example "of $500.00 - $150.00 -&gt; Credit CM-1042").
-2. Otherwise it reads exactly "of {full amount} - {excess} will be credited".
-3. {full amount} is the payment's or deposit's full amount; {excess} is the full amount minus the amount applied to this invoice.
-4. The em dash and the arrow are literal separator characters, not subtraction.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R5, read on 25 August 2026.
+          <t xml:space="preserve">1. A sub-line is shown beneath any payment or deposit whose amount applied to this invoice is less than its full amount - this is not limited to deposits and includes a regular payment spread across more than one invoice. It gates on applied being less than the full amount, never on whether the row is a deposit.
+2. When the excess has become a customer-account credit with a number, the sub-line reads exactly "of {full amount} — {excess} → Credit {credit number}" (for example "of $500.00 — $150.00 → Credit CM-1042").
+3. Otherwise it reads exactly "of {full amount} — {excess} will be credited".
+4. {full amount} is the payment's or deposit's full amount; {excess} is the full amount minus the amount applied to this invoice.
+5. The em dash and the arrow are literal separator characters, not subtraction.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3071,7 +3073,7 @@
 2. Balance equals the Total minus all applied payments (any method), applied deposits, and applied customer-account credits.
 3. Balance is floored at $0.00: an overpaid invoice shows "Balance" with "$0.00" - never a negative amount and never a hidden row.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R6, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-R6, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3126,7 +3128,7 @@
 4. The banner shows a fixed status pill: exactly "PAID IN FULL" when the invoice is fully paid at generation time, otherwise exactly "PARTIALLY PAID".
 5. The banner title reads exactly "Payment Receipt (Batch) - Payments by ShopView" when every listed payment was part of a batch, otherwise exactly "Payment Receipt - Payments by ShopView".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-R8, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-R8, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3181,7 +3183,7 @@
 5. In a batch, each payment carries a "Payment X of Y - Batch" marker.
 6. "Date / Time" reads in the format "Jan 5, 2026 - 2:41 PM MST" (date, then time with timezone).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, sections S8-R9 and G-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, sections S8-R9 and G-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3232,7 +3234,7 @@
           <t xml:space="preserve">1. A payment row whose amount is $0.00 is not shown.
 2. When no payments, deposits or customer-account credits have been applied, the Payments heading shows with no rows and the Balance equals the Total.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, sections S8-R7 and S8-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, sections S8-R7 and S8-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3283,7 +3285,7 @@
           <t xml:space="preserve">1. When the invoice has no portal-processed payment, the paid banner is not shown - a shop-recorded payment never produces the banner.
 2. An Invoice PDF generated in the shop app shows no banner in any case.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 39, section S8-N2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9147 (Story 8, Paid Banner, Payments and Balance) and the Invoice UI Refresh specification version 45, section S8-N2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3334,7 +3336,7 @@
           <t xml:space="preserve">1. Each document shows the shop's configured disclaimer text, with no heading above it.
 2. The disclaimer is identical on every document that carries it.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, section S9-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 45, section S9-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3386,7 +3388,7 @@
 2. The three lines are identical on every document that carries the area.
 3. The signature area contains no authorization or acknowledgment sentence - only the three lines.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, sections S9-R2 and S9-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 45, sections S9-R2 and S9-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3437,7 +3439,7 @@
           <t xml:space="preserve">1. The footer shows the shop's tax identifier exactly as the shop entered it.
 2. No label is added in front of it (the shop types its own label into the field).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, section S9-R4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 45, section S9-R4, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3488,7 +3490,7 @@
           <t xml:space="preserve">1. When the shop has no configured disclaimer, the disclaimer area is not shown.
 2. When the shop has no tax identifier configured, the footer tax identifier is not shown.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 39, sections S9-N1 and S9-N2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9148 (Story 9, Disclaimer, Signature and Footer) and the Invoice UI Refresh specification version 45, sections S9-N1 and S9-N2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3538,7 +3540,7 @@
         <is>
           <t xml:space="preserve">1. The Estimate and Invoice carry the same content, differing only in: the document label, the dates, the work-section heading, the headline figure label, and the presence of the Paid banner and the Payments and Balance sections on the Invoice.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 45, section S10-R1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3592,7 +3594,7 @@
 4. No validity or expiry date is shown; no due-date line is shown.
 5. The signature area's "Date" line is unaffected.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 45, section S10-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3644,7 +3646,7 @@
 2. The boxed headline figure is labeled "Balance".
 3. The masthead shows "Invoice date: {date}" and "Due date: {date}".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 45, section S10-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3698,7 +3700,7 @@
 4. If a later change (payment reversal, voided credit, or edit) makes the Balance greater than $0.00, the invoice is no longer fully paid and "Due date: {date}" returns.
 5. A paid date earlier than the invoice date (for example a deposit collected before invoicing) is shown as-is.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-R4, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 45, section S10-R4, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3749,7 +3751,7 @@
           <t xml:space="preserve">1. An Invoice with no due date set shows "Invoice date: {date}" and no "Due date" line (the old quirk of rendering a null due date as today's date is retired).
 2. When such an invoice becomes fully paid, "Paid date: {date}" is shown.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 39, section S10-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9149 (Story 10, Estimate and Invoice Specifics) and the Invoice UI Refresh specification version 45, section S10-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3801,7 +3803,7 @@
 2. The masthead shows "Issue date: {date}".
 3. The masthead shows no money figure and no boxed headline figure.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R1 and S1-R6, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, sections S11-R1 and S1-R6, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3853,7 +3855,7 @@
 2. Every other address rule applies to it unchanged (name always shown, address fields hide when empty).
 3. Remit Payment To never appears on the Credit Invoice, so the Credit To block is always full width.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R2, S2-R1 and S2-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, sections S11-R2, S2-R1 and S2-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3906,7 +3908,7 @@
 3. Invoice Number shows the originating invoice's full document number (for example "").
 4. For an account-level credit with no origin invoice, the whole Invoice Number column is hidden.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, section S11-R3, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, section S11-R3, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -3961,7 +3963,7 @@
 5. Totals are negative, formatted with a leading minus (for example "-$100.00") - not the parentheses convention used for discounts.
 6. A money-only line's Description comes from the credit's reason if entered, otherwise the memo text, otherwise "Refund".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R4 and S11-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, sections S11-R4 and S11-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4012,7 +4014,7 @@
           <t xml:space="preserve">1. The restocking fee reduces the credit: quantity -2 at rate $50.00 with a $10.00 restocking fee produces Total -$90.00.
 2. For a money-only line, Total is the credited amount.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, section S11-R5, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, section S11-R5, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4062,12 +4064,14 @@
         <is>
           <t xml:space="preserve">1. The totals block shows rows labeled exactly: "Subtotal" (sum of item totals, negative), "Tax" (one row; negative when tax applies, "$0.00" when none), "Total Credit" (negative, the document's key figure), "Payments", and "Balance".
 2. Unapplied: Payments shows the label with no rows; Balance shows the full credit amount, positive (its open balance).
-3. Partially applied: Payments shows the label with no rows; Balance shows the open balance, positive (original minus amounts applied to invoices).
+3. Partially applied: Payments shows the label with no rows; Balance shows the open balance, positive (original credit total minus amounts refunded minus amounts applied to invoices).
 4. Applied: Payments shows the label with no rows; Balance reads $0.00.
 5. Refunded: one row per refund payment reading "{date} - {method}" with the refunded amount (negative); Balance reads $0.00 once fully consumed, otherwise the open balance, positive.
 6. Voided: Payments shows the label with no rows; Balance reads $0.00.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R6 and S11-R6a, read on 25 August 2026.
+7. On the Credit Invoice, "Balance" is the credit's open balance — the original credit total minus amounts refunded minus amounts applied to invoices — shown positive, reading $0.00 once nothing remains or the credit is voided; it does not follow the Invoice's Total-minus-payments formula.
+8. A credit that is both partially refunded and partially applied takes the "Partially applied" status (one of the five states, not a new one), and its refund rows still list in the Payments section.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, sections S11-R6 and S11-R6a, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4118,7 +4122,7 @@
           <t xml:space="preserve">1. The Credit Invoice shows the shop's configured disclaimer.
 2. It shows the standard signature area with the three lines "Customer Signature", "Printed Name", and "Date".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 39, sections S11-R7 and S9-R2, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9150 (Story 11, Credit Invoice) and the Invoice UI Refresh specification version 45, sections S11-R7 and S9-R2, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4168,7 +4172,7 @@
         <is>
           <t xml:space="preserve">1. The document layout follows the Design Document exactly: masthead with the shop letterhead left, the shop logo center, and the document block right over a 2px ink rule; a bordered Addresses row; the asset band; the order reference chips; numbered work lines; the "Summary" break bar; a two-column tail with the disclaimer left and the totals right; the boxed headline figure; the three-line signature row; the single-line footer.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R1, and the Design Document, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R1, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4216,10 +4220,10 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The only colours on any document are: ink #121926, body text #364152, muted text #697586, faint labels #9AA4B2, hairlines #E3E8EF, row dividers #EEF2F6, accent #257CFF, negative #B42318, paper #FFFFFF.
-2. No colour outside this closed set appears.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R2, and the Design Document, read on 25 August 2026.
+          <t xml:space="preserve">1. The only colours on the light printed document are: ink #121926, body text #364152, muted text #697586, faint labels #9AA4B2, hairlines #E3E8EF, row dividers #EEF2F6, paid-banner surface #F8FAFC, accent #257CFF, negative #B42318, paper #FFFFFF.
+2. No colour outside this set appears on the printed document; the print and black-and-white output adds only the inks S12-R5 lists, and the Design Document's demo chrome and dark-mode preview are not part of any document.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R2, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4268,9 +4272,10 @@
       <c r="G74" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The accent #257CFF appears only on the work line numbers and on the word "ShopView" in the footer.
-2. Nothing else on the document uses the accent.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R3, and the Design Document, read on 25 August 2026.
+2. On the Parts Sale document, which has no numbered work lines, the accent appears only on the word "ShopView" in the footer.
+3. Nothing else on the document uses the accent.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R3, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4318,11 +4323,11 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The typeface is Inter with a system sans-serif fallback.
-2. Weight 400 for body text; 600 and 700 for emphasis and totals; 750 for the in-job section labels; 800 for the shop name, the document label, the headline figure, and the line numbers.
+          <t xml:space="preserve">1. The typeface is Inter with a system sans-serif fallback, applied identically on screen and in PDF output, so the on-screen preview and the PDF wrap line for line.
+2. Weight 400 for body text; 600 and 700 for emphasis and totals; 700 for the in-job section labels; 800 for the shop name, the document label, the headline figure, and the line numbers.
 3. Uppercase micro-labels carry letterspacing as in the Design Document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R4, and the Design Document, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R4, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4374,7 +4379,7 @@
 2. Text smaller than 10px renders no lighter than #364152.
 3. Hairline rules render no lighter than #CDD5DF.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R5, and the Design Document, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R5, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4425,7 +4430,7 @@
           <t xml:space="preserve">1. Every document is fully legible printed in grayscale.
 2. Colour is never the only signal: credit amounts also carry the leading minus, and discounts also carry parentheses.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R6, and the Design Document, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R6, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4473,11 +4478,11 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. The Design Document's control strips (the document and field toggles, the settings menu, the POC badge, the theme controls) do not appear on any real document.
+          <t xml:space="preserve">1. The Design Document's control strips (the document and field toggles, the settings menu, the theme controls) do not appear on any real document.
 2. Only the white sheet is the document.
 3. The PDF output carries no drop shadow and no rounded sheet corners (those are screen-prototype presentation only).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, sections S12-R7 and S12-N1, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, sections S12-R7 and S12-N1, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4531,7 +4536,7 @@
 4. The "Labor" and "Parts" sub-section labels carry no underline rule.
 5. When a line has fee or discount adjustment rows, the row divider follows the line's last adjustment row - never between the line and its adjustments - so the line and its adjustments read as one group.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R8, and the Design Document, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R8, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4580,11 +4585,11 @@
       <c r="G80" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The document section label ("Work Summary" / "Work Performed" / "Parts") is 11px weight 700 in muted ink #697586.
-2. "Scope of work" is 10px weight 750 in body ink #364152.
-3. The in-job "Labor" and "Parts" labels are 10.5px weight 750 in full ink #121926.
+2. "Scope of work" is 10px weight 700 in body ink #364152.
+3. The in-job "Labor" and "Parts" labels are 10.5px weight 700 in full ink #121926.
 4. All three sit visually below the 16px weight-700 job titles, with letterspacing per the Design Document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 39, section S12-R9, and the Design Document, read on 25 August 2026.
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R9, and the Design Document, read on 31 August 2026.
 AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
 </t>
         </is>
@@ -4600,414 +4605,524 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
+          <t>Multi-page document uses standard page-break behaviour</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Document Visual Standard</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to ShopView.
+2. You can generate a document long enough to span more than one page (a work order with many work lines), on screen and as a PDF.</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>1. Generate a multi-page document.
+2. Look at the top of every page after the first.
+3. Check the totals block, a work line together with its own footer, the signature row, and any single row that falls near a page boundary.</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. Long documents paginate using standard, globally accepted page-break behaviour, not custom pagination.
+2. Every page after the first opens with a single identification line: the shop location's name on the left and the document number on the right (for example "Heavy Duty - 9919" on the left and "Invoice: INV-S2-4802" on the right).
+3. The full masthead does not repeat on later pages.
+4. The totals block is not split across a page break.
+5. A work line and its own footer stay together on the same page.
+6. The signature row does not land alone on a final page.
+7. No single row is orphaned by itself on a page.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R10, and the Design Document, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/31/2026
+</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>SV-9151 (S12-R10)</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="inlineStr"/>
+      <c r="J81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>On-screen document fits the viewport; wide elements scroll in their own container</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>Document Visual Standard</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>1. You are signed in to ShopView.
+2. You can view a document on screen and narrow the browser viewport, ideally with a document that contains a wide element such as a wide table.</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>1. Open a document on screen and narrow the viewport.
+2. Check whether any content is clipped.
+3. Find an element wider than the viewport (for example a wide table) and check how it behaves.</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. On screen the document fits within the viewport with no content clipped.
+2. Any element wider than the viewport (for example a wide table) scrolls horizontally within its own container, rather than clipping or forcing the whole page to scroll sideways.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9151 (Story 12, Document Visual Standard) and the Invoice UI Refresh specification version 45, section S12-R11, and the Design Document, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/31/2026
+</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>SV-9151 (S12-R11)</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="inlineStr"/>
+      <c r="J82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
           <t>Parts Sale documents behave as the Estimate/Invoice except as stated</t>
         </is>
       </c>
-      <c r="B81" s="2" t="inlineStr">
+      <c r="B83" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C81" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D81" s="2" t="inlineStr">
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E81" s="2" t="inlineStr">
+      <c r="E83" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. You can generate a Parts Sale Estimate and a Parts Sale Invoice.</t>
         </is>
       </c>
-      <c r="F81" s="2" t="inlineStr">
+      <c r="F83" s="2" t="inlineStr">
         <is>
           <t>1. Generate a Parts Sale Estimate and a Parts Sale Invoice.
 2. Check masthead, dates, addresses, Remit Payment To, asset section, financial summary, payments/Balance, paid banner, disclaimer/signature, and visual standard.</t>
         </is>
       </c>
-      <c r="G81" s="2" t="inlineStr">
+      <c r="G83" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The Parts Sale Estimate behaves as the Estimate, and the Parts Sale Invoice as the Invoice, throughout the spec: masthead and date labels (including "Estimate date" and the Due/Paid date swap), addresses and Remit Payment To, asset section, financial summary, payments and Balance, the paid banner rule, disclaimer and signature, and the visual standard - except as Story 13 states.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R1, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H81" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-R1, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R1)</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr"/>
-      <c r="J81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="inlineStr">
+      <c r="I83" s="2" t="inlineStr"/>
+      <c r="J83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>Parts Sale body is a single flat 'Parts' section, no jobs</t>
         </is>
       </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E82" s="2" t="inlineStr">
+      <c r="E84" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. A Parts Sale Estimate or Invoice exists with several part lines.</t>
         </is>
       </c>
-      <c r="F82" s="2" t="inlineStr">
+      <c r="F84" s="2" t="inlineStr">
         <is>
           <t>1. Generate the Parts Sale document.
 2. Read the body section.</t>
         </is>
       </c>
-      <c r="G82" s="2" t="inlineStr">
+      <c r="G84" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The body is a single section headed "Parts".
 2. It shows flat part lines, each with part number, description, quantity, rate, and amount.
 3. There are no job blocks, no "Scope of work", no Labor section, and no Declined Work section on a parts sale document.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R2, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H82" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-R2, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R2)</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr"/>
-      <c r="J82" s="2" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="inlineStr">
+      <c r="I84" s="2" t="inlineStr"/>
+      <c r="J84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>Parts Sale line-level fees/discounts render as on the Invoice</t>
         </is>
       </c>
-      <c r="B83" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C83" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D83" s="2" t="inlineStr">
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E83" s="2" t="inlineStr">
+      <c r="E85" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. A Parts Sale document has a part line with a line-level fee or discount.</t>
         </is>
       </c>
-      <c r="F83" s="2" t="inlineStr">
+      <c r="F85" s="2" t="inlineStr">
         <is>
           <t>1. Generate the Parts Sale document.
 2. Read the part line that has an adjustment.</t>
         </is>
       </c>
-      <c r="G83" s="2" t="inlineStr">
+      <c r="G85" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Line-level fees and discounts render exactly as on the Invoice: indented under their part line.
 2. The row divider follows the part's last adjustment row, rather than sitting between the part and its adjustments.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, sections S13-R3 and S12-R8, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H83" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, sections S13-R3 and S12-R8, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R3; S12-R8)</t>
         </is>
       </c>
-      <c r="I83" s="2" t="inlineStr"/>
-      <c r="J83" s="2" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="inlineStr">
+      <c r="I85" s="2" t="inlineStr"/>
+      <c r="J85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
         <is>
           <t>Parts Sale document number keeps parts-sale numbering</t>
         </is>
       </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E84" s="2" t="inlineStr">
+      <c r="E86" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. You can generate a Parts Sale Estimate and Invoice with parts-sale numbering.</t>
         </is>
       </c>
-      <c r="F84" s="2" t="inlineStr">
+      <c r="F86" s="2" t="inlineStr">
         <is>
           <t>1. Generate the Parts Sale Estimate and read its masthead label.
 2. Generate the Parts Sale Invoice and read its masthead label.</t>
         </is>
       </c>
-      <c r="G84" s="2" t="inlineStr">
+      <c r="G86" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The document number uses the parts-sale numbering through the existing document numbering.
 2. For example the Estimate reads "Estimate: EST-P2-1088" and the Invoice reads "Invoice: INV-P2-1088".
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R4, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H84" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-R4, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R4)</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr"/>
-      <c r="J84" s="2" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="inlineStr">
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>Parts Sale reference fields drop Work Order and Approval Code</t>
         </is>
       </c>
-      <c r="B85" s="2" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E85" s="2" t="inlineStr">
+      <c r="E87" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. You can generate a Parts Sale document with a Customer PO, Terms, and an Authorizer set.</t>
         </is>
       </c>
-      <c r="F85" s="2" t="inlineStr">
+      <c r="F87" s="2" t="inlineStr">
         <is>
           <t>1. Generate the Parts Sale document.
 2. Read the order reference fields area.</t>
         </is>
       </c>
-      <c r="G85" s="2" t="inlineStr">
+      <c r="G87" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The Work Order field and the Approval Code field are not shown on a parts sale document.
 2. Customer PO and Terms are unchanged (Terms always shows).
 3. Authorizer follows the parts-sale Authorizer treatment (S13-R6).
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R5, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H85" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-R5, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H87" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R5)</t>
         </is>
       </c>
-      <c r="I85" s="2" t="inlineStr"/>
-      <c r="J85" s="2" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="inlineStr">
+      <c r="I87" s="2" t="inlineStr"/>
+      <c r="J87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
         <is>
           <t>Parts sale receives the Authorizer treatment (net-new)</t>
         </is>
       </c>
-      <c r="B86" s="2" t="inlineStr">
+      <c r="B88" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C86" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D86" s="2" t="inlineStr">
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E86" s="2" t="inlineStr">
+      <c r="E88" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView with access to parts sales.
 2. A parts sale exists for a customer with 'Approves Work' contacts.</t>
         </is>
       </c>
-      <c r="F86" s="2" t="inlineStr">
+      <c r="F88" s="2" t="inlineStr">
         <is>
           <t>1. Open the parts sale record and find the Authorizer field.
 2. Select an authorizer from the offered list, then invoice the parts sale and try to change it.
 3. Generate the Parts Sale document and read the Authorizer reference field.</t>
         </is>
       </c>
-      <c r="G86" s="2" t="inlineStr">
+      <c r="G88" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The parts sale has an Authorizer field offering the customer's "Approves Work" contacts, empty by default, filled by the user.
 2. It is locked once the parts sale is invoiced.
-3. When set, the authorizer's name prints in the document's Authorizer reference field.
----
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R6, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H86" s="2" t="inlineStr">
+3. If that invoice is voided or reversed, the Authorizer becomes editable again (mirrors S3-R8).
+4. When set, the authorizer's name prints in the document's Authorizer reference field.
+---
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-R6, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R6)</t>
         </is>
       </c>
-      <c r="I86" s="2" t="inlineStr"/>
-      <c r="J86" s="2" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="inlineStr">
+      <c r="I88" s="2" t="inlineStr"/>
+      <c r="J88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
         <is>
           <t>Parts Sale financial summary shows no Labor and no Shop supplies row</t>
         </is>
       </c>
-      <c r="B87" s="2" t="inlineStr">
+      <c r="B89" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C87" s="2" t="inlineStr">
-        <is>
-          <t>Functional</t>
-        </is>
-      </c>
-      <c r="D87" s="2" t="inlineStr">
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Functional</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E87" s="2" t="inlineStr">
+      <c r="E89" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. A Parts Sale Invoice exists with parts charges, adjustments, tax and payments.</t>
         </is>
       </c>
-      <c r="F87" s="2" t="inlineStr">
+      <c r="F89" s="2" t="inlineStr">
         <is>
           <t>1. Generate the Parts Sale Invoice.
 2. Read the financial summary.</t>
         </is>
       </c>
-      <c r="G87" s="2" t="inlineStr">
+      <c r="G89" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The financial summary shows no "Labor" row and no "Shop supplies" row.
 2. The "Parts" row, the adjustment rows, "Subtotal", "Tax", "Total", "Payments", and "Balance" are identical to the Invoice.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-R7, read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H87" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-R7, read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-R7)</t>
         </is>
       </c>
-      <c r="I87" s="2" t="inlineStr"/>
-      <c r="J87" s="2" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="inlineStr">
+      <c r="I89" s="2" t="inlineStr"/>
+      <c r="J89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>Batch and imported invoices are out of scope (kept on current templates)</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>Parts Sale Estimate and Invoice</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="D88" s="2" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="E88" s="2" t="inlineStr">
+      <c r="E90" s="2" t="inlineStr">
         <is>
           <t>1. You are signed in to ShopView.
 2. You can generate a batch invoice and an imported invoice.</t>
         </is>
       </c>
-      <c r="F88" s="2" t="inlineStr">
+      <c r="F90" s="2" t="inlineStr">
         <is>
           <t>1. Generate a batch invoice and an imported invoice.
 2. Confirm they are not restyled by this project.</t>
         </is>
       </c>
-      <c r="G88" s="2" t="inlineStr">
+      <c r="G90" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Batch invoices and imported invoices are not part of Story 13 or this spec.
 2. They keep their current templates until the follow-up ticket (SV-9193) ships.
 3. Restyling shared template partials must not half-restyle these deferred templates.
 ---
-This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 39, section S13-N1, and story SV-9193 (deferred), read on 25 August 2026.
-AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
-</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
+This is the expected behaviour as per epic SV-8218 and story SV-9195 (Story 13, Parts Sale Estimate and Invoice) and the Invoice UI Refresh specification version 45, section S13-N1, and story SV-9193 (deferred), read on 31 August 2026.
+AUTOMATION: Not available on Build to test Yet - Last checked 8/21/2026
+</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
         <is>
           <t>SV-9195 (S13-N1); SV-9193 (deferred)</t>
         </is>
       </c>
-      <c r="I88" s="2" t="inlineStr"/>
-      <c r="J88" s="2" t="inlineStr"/>
+      <c r="I90" s="2" t="inlineStr"/>
+      <c r="J90" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>